<commit_message>
updated dry bean files and quarto book
</commit_message>
<xml_diff>
--- a/drybeans/data_final/production_cost.xlsx
+++ b/drybeans/data_final/production_cost.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">sheet_name</t>
   </si>
@@ -21,91 +21,64 @@
     <t xml:space="preserve">description</t>
   </si>
   <si>
-    <t xml:space="preserve">notes</t>
-  </si>
-  <si>
     <t xml:space="preserve">source</t>
   </si>
   <si>
     <t xml:space="preserve">production_cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Mean and standard deviation for cost of production per acre and hectare for dry bean and soybean growers. Costs are by crop, location (in NY/outside NY), scale (under/over $M), organic, and MWBE).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing data means there were no farms of that type in the data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restricted access census of agriculture and crop budgets. See Quarto file for more information.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">variable_name</t>
+    <t xml:space="preserve">Mean and standard deviation for cost of production per acre and hectare for dry bean and soybean growers. Costs are by crop, scale (under/over $M), organic, and MWBE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restricted access Census of Agriculture and crop budgets. See Quarto file for more information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">crop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sales_class_agg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mwbe_fct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">organic_fct</t>
   </si>
   <si>
     <t xml:space="preserve">production_cost_acre_mean</t>
   </si>
   <si>
-    <t xml:space="preserve">production_cost_acre_se</t>
+    <t xml:space="preserve">production_cost_acre_sd</t>
   </si>
   <si>
     <t xml:space="preserve">production_cost_hectare_mean</t>
   </si>
   <si>
-    <t xml:space="preserve">production_cost_hectare_se</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_more_mill_nonmwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_more_mill_mwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_less_mill_nonmwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_less_mill_mwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_more_mill_nonmwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_more_mill_mwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_less_mill_nonmwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_less_mill_mwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_drybean_outsideNY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_more_mill_nonmwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_more_mill_mwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_less_mill_nonmwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_less_mill_mwbe_conv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_more_mill_nonmwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_more_mill_mwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_less_mill_nonmwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_less_mill_mwbe_org</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cost_of_production_soy_outsideNY</t>
+    <t xml:space="preserve">production_cost_hectare_sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drybeans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCFI $1 million or more</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MWBE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No organic sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organic sales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not MWBE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCFI less than $1 million</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soybeans</t>
   </si>
 </sst>
 </file>
@@ -444,22 +417,16 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -475,270 +442,445 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="n">
-        <v>518.4375</v>
-      </c>
-      <c r="C2" t="n">
-        <v>155.859375</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1281.0590625</v>
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
       </c>
       <c r="E2" t="n">
-        <v>385.128515625</v>
+        <v>451.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>42.7205</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1115.6565</v>
+      </c>
+      <c r="H2" t="n">
+        <v>105.5623555</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3"/>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="n">
+        <v>485.1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>45.8997</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1198.6821</v>
+      </c>
+      <c r="H3" t="n">
+        <v>113.4181587</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="n">
-        <v>360.9375</v>
-      </c>
-      <c r="C4" t="n">
-        <v>131.25</v>
-      </c>
-      <c r="D4" t="n">
-        <v>891.8765625</v>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
       </c>
       <c r="E4" t="n">
-        <v>324.31875</v>
+        <v>740.526315789474</v>
+      </c>
+      <c r="F4" t="n">
+        <v>70.0678947368421</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1829.84052631579</v>
+      </c>
+      <c r="H4" t="n">
+        <v>173.137767894737</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="n">
-        <v>393.75</v>
-      </c>
-      <c r="C5" t="n">
-        <v>147.65625</v>
-      </c>
-      <c r="D5" t="n">
-        <v>972.95625</v>
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>364.85859375</v>
+        <v>550.62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>52.09914</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1360.58202</v>
+      </c>
+      <c r="H5" t="n">
+        <v>128.73697494</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
+      <c r="E6" t="n">
+        <v>509.636842105263</v>
+      </c>
+      <c r="F6" t="n">
+        <v>48.221352631579</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1259.31263684211</v>
+      </c>
+      <c r="H6" t="n">
+        <v>119.154962352632</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
+      <c r="E7" t="n">
+        <v>988.68</v>
+      </c>
+      <c r="F7" t="n">
+        <v>93.54796</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2443.02828</v>
+      </c>
+      <c r="H7" t="n">
+        <v>231.15700916</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="n">
-        <v>656.25</v>
-      </c>
-      <c r="C8" t="n">
-        <v>164.0625</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1621.59375</v>
+      <c r="D8" t="s">
+        <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>405.3984375</v>
+        <v>342.189473684211</v>
+      </c>
+      <c r="F8" t="n">
+        <v>32.3776421052632</v>
+      </c>
+      <c r="G8" t="n">
+        <v>845.550189473684</v>
+      </c>
+      <c r="H8" t="n">
+        <v>80.0051536421053</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="n">
+        <v>314.034</v>
+      </c>
+      <c r="F9" t="n">
+        <v>29.713598</v>
+      </c>
+      <c r="G9" t="n">
+        <v>775.978014</v>
+      </c>
+      <c r="H9" t="n">
+        <v>73.422300658</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="n">
-        <v>471.83</v>
-      </c>
-      <c r="C10" t="n">
-        <v>43.7614573569026</v>
-      </c>
-      <c r="D10" t="n">
-        <v>1165.89193</v>
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>108.134561128906</v>
+        <v>827.843342036554</v>
+      </c>
+      <c r="F10" t="n">
+        <v>640.21753827118</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2045.60089817232</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1581.97753706808</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="n">
-        <v>815.094339622641</v>
-      </c>
-      <c r="C11" t="n">
-        <v>37.7358490566038</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2014.09811320755</v>
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
       </c>
       <c r="E11" t="n">
-        <v>93.2452830188679</v>
+        <v>829.724804177546</v>
+      </c>
+      <c r="F11" t="n">
+        <v>550.939151436031</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2050.24999112272</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1361.37064319843</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="n">
-        <v>815.094339622641</v>
-      </c>
-      <c r="C12" t="n">
-        <v>75.4716981132076</v>
-      </c>
-      <c r="D12" t="n">
-        <v>2014.09811320755</v>
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
       </c>
       <c r="E12" t="n">
-        <v>186.490566037736</v>
+        <v>832.860574412533</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1661.91500019866</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2057.99847937337</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4106.59196549089</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="n">
-        <v>822.641509433962</v>
-      </c>
-      <c r="C13" t="n">
-        <v>15.0943396226415</v>
-      </c>
-      <c r="D13" t="n">
-        <v>2032.74716981132</v>
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>17</v>
       </c>
       <c r="E13" t="n">
-        <v>37.2981132075472</v>
+        <v>843.365404699739</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2321.98715045836</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2083.95591501305</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5737.63024878261</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" t="n">
-        <v>816.603773584906</v>
-      </c>
-      <c r="C14" t="n">
-        <v>22.6415094339623</v>
-      </c>
-      <c r="D14" t="n">
-        <v>2017.8279245283</v>
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>55.9471698113208</v>
+        <v>863.198829788581</v>
+      </c>
+      <c r="F14" t="n">
+        <v>667.559913553556</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2132.96430840758</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1649.54054639084</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15"/>
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15"/>
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" t="n">
+        <v>865.160645310828</v>
+      </c>
+      <c r="F15" t="n">
+        <v>574.468630301912</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2137.81195456306</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1419.51198547602</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16"/>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" t="n">
+        <v>868.430337847906</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1732.89197428398</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2145.89136482218</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4281.97606845572</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" t="n">
-        <v>679.245283018868</v>
-      </c>
-      <c r="C17" t="n">
-        <v>45.2830188679245</v>
-      </c>
-      <c r="D17" t="n">
-        <v>1678.41509433962</v>
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>18</v>
       </c>
       <c r="E17" t="n">
-        <v>111.894339622642</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" t="n">
-        <v>1358.49056603774</v>
-      </c>
-      <c r="C18" t="n">
-        <v>528.301886792453</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3356.83018867925</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1305.43396226415</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19"/>
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
+        <v>879.383807847117</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2421.15444949882</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2172.95738919023</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5982.6726447116</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>